<commit_message>
first round report done. Partial reproduction due to README issues and minor discrepancies
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/damandhaliwal/Documents/Research Work/JPE/Replications/JPE-Castro-Vincenzi-20240641-R1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F50C8F0-0FD7-C549-B265-C4B589168668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="17080" windowHeight="27480" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="158">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -45,7 +45,469 @@
     <t>Line Number</t>
   </si>
   <si>
-    <t>In-text numbers</t>
+    <t>BEA_KLEMS.do</t>
+  </si>
+  <si>
+    <t>BEA-BLS_klems_clean.dta</t>
+  </si>
+  <si>
+    <t>agg_fred_prices.do</t>
+  </si>
+  <si>
+    <t>fred_prices.dta</t>
+  </si>
+  <si>
+    <t>agg_labour_shares.do</t>
+  </si>
+  <si>
+    <t>agglabshr.dta</t>
+  </si>
+  <si>
+    <t>bea_county.do</t>
+  </si>
+  <si>
+    <t>bea_county_gdp.dta
+bea_county_otheraggdata.dta</t>
+  </si>
+  <si>
+    <t>bea_historical.do</t>
+  </si>
+  <si>
+    <t>bea_historical.dta</t>
+  </si>
+  <si>
+    <t>build_censuscr_raw.do</t>
+  </si>
+  <si>
+    <t>censuscr_97-02-07-12_n6.dta</t>
+  </si>
+  <si>
+    <t>cep_cleaned.do</t>
+  </si>
+  <si>
+    <t>comtrade_lit_energysafe_gassplice_cepiisplice11.dta
+Commodity_Prices_HS96.dta
+Commodity_Prices_Weight_comtrade_new.dta</t>
+  </si>
+  <si>
+    <t>concentration.do</t>
+  </si>
+  <si>
+    <t>concentration.dta</t>
+  </si>
+  <si>
+    <t>create_shares.do</t>
+  </si>
+  <si>
+    <t>IOLinkages.dta</t>
+  </si>
+  <si>
+    <t>create_ss_dataset.do</t>
+  </si>
+  <si>
+    <t>mainregfile.dta</t>
+  </si>
+  <si>
+    <t>create_ss_instrument.do</t>
+  </si>
+  <si>
+    <t>shiftshare_ct.dta</t>
+  </si>
+  <si>
+    <t>crosscountry_iv.do</t>
+  </si>
+  <si>
+    <t>wiod_io_shares_2000.dta
+comtrade_wiod_prices.dta
+crosscountry_iv.dta</t>
+  </si>
+  <si>
+    <t>crosscountry_panel_build.do</t>
+  </si>
+  <si>
+    <t>klems_panel_2025.dta</t>
+  </si>
+  <si>
+    <t>crosscountry_panel_finalize.do</t>
+  </si>
+  <si>
+    <t>crosscountry_iv_merge.dta
+crosscountry_panel.dta</t>
+  </si>
+  <si>
+    <t>disaster_iv_construct.do</t>
+  </si>
+  <si>
+    <t>disaster_iv_data.dta</t>
+  </si>
+  <si>
+    <t>exchange_rates.do</t>
+  </si>
+  <si>
+    <t>fx.dta</t>
+  </si>
+  <si>
+    <t>model_inputs.do</t>
+  </si>
+  <si>
+    <t>subsector_data.csv
+data_manufacturing.csv</t>
+  </si>
+  <si>
+    <t>oilprices.do</t>
+  </si>
+  <si>
+    <t>oilprices.dta</t>
+  </si>
+  <si>
+    <t>qcew_panels.do</t>
+  </si>
+  <si>
+    <t>QCEW_naics4_panel.dta
+QCEW_naics2_panel.dta</t>
+  </si>
+  <si>
+    <t>regional.do</t>
+  </si>
+  <si>
+    <t>regional.dta</t>
+  </si>
+  <si>
+    <t>trade.do</t>
+  </si>
+  <si>
+    <t>imports_1989-2018_naics.dta
+exports_1989-2018_naics.dta</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>do/figures/fig1.do</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>Supplied</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>do/figures/fig3.do</t>
+  </si>
+  <si>
+    <t>120, 175, 183</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>do/figures/fig4.do</t>
+  </si>
+  <si>
+    <t>120, 129</t>
+  </si>
+  <si>
+    <t>Figure 5</t>
+  </si>
+  <si>
+    <t>do/figures/fig5.do</t>
+  </si>
+  <si>
+    <t>103, 158, 173</t>
+  </si>
+  <si>
+    <t>Figure 6</t>
+  </si>
+  <si>
+    <t>do/figures/fig6.do</t>
+  </si>
+  <si>
+    <t>61, 70</t>
+  </si>
+  <si>
+    <t>Figure 7</t>
+  </si>
+  <si>
+    <t>do/figures/fig7.do</t>
+  </si>
+  <si>
+    <t>180, 360</t>
+  </si>
+  <si>
+    <t>Figure 8</t>
+  </si>
+  <si>
+    <t>quant_model/plots.jl</t>
+  </si>
+  <si>
+    <t>56, 57, 58</t>
+  </si>
+  <si>
+    <t>Figure 9</t>
+  </si>
+  <si>
+    <t>111-115, 133</t>
+  </si>
+  <si>
+    <t>Figure B.1</t>
+  </si>
+  <si>
+    <t>do/figures/figB1.do</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>Figure C.1</t>
+  </si>
+  <si>
+    <t>do/figures/figC1.do</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>Figure C.2</t>
+  </si>
+  <si>
+    <t>do/figures/figC2.do</t>
+  </si>
+  <si>
+    <t>222</t>
+  </si>
+  <si>
+    <t>Figure C.3</t>
+  </si>
+  <si>
+    <t>do/figures/figC3.do</t>
+  </si>
+  <si>
+    <t>77, 104</t>
+  </si>
+  <si>
+    <t>Figure C.4</t>
+  </si>
+  <si>
+    <t>do/figures/figC4.do</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>Figure C.5</t>
+  </si>
+  <si>
+    <t>do/figures/figC5.do</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>Figure E.1</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>Figure E.2</t>
+  </si>
+  <si>
+    <t>134</t>
+  </si>
+  <si>
+    <t>Figure E.3</t>
+  </si>
+  <si>
+    <t>216</t>
+  </si>
+  <si>
+    <t>Figure F.1</t>
+  </si>
+  <si>
+    <t>do/figures/fig_crosscountry.do</t>
+  </si>
+  <si>
+    <t>77, 114</t>
+  </si>
+  <si>
+    <t>Figure F.2</t>
+  </si>
+  <si>
+    <t>319, 331</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>do/tables/tab1.do</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>do/tables/tab2.do</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>do/tables/tab3.do</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>do/tables/tab4.do</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>Table B.1</t>
+  </si>
+  <si>
+    <t>Table C.1</t>
+  </si>
+  <si>
+    <t>do/tables/tabC1.do</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>Table C.2</t>
+  </si>
+  <si>
+    <t>do/tables/tabC2.do</t>
+  </si>
+  <si>
+    <t>Table C.3</t>
+  </si>
+  <si>
+    <t>do/tables/tabC3.do</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>Table C.4</t>
+  </si>
+  <si>
+    <t>do/tables/tabC4.do</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>Table C.5</t>
+  </si>
+  <si>
+    <t>do/tables/tabC5.do</t>
+  </si>
+  <si>
+    <t>96</t>
+  </si>
+  <si>
+    <t>Table C.6</t>
+  </si>
+  <si>
+    <t>do/tables/tabC6.do</t>
+  </si>
+  <si>
+    <t>Table C.7</t>
+  </si>
+  <si>
+    <t>do/tables/tabC7.do</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>Table C.8</t>
+  </si>
+  <si>
+    <t>do/tables/tabC8.do</t>
+  </si>
+  <si>
+    <t>Table C.9</t>
+  </si>
+  <si>
+    <t>do/tables/tabC9.do</t>
+  </si>
+  <si>
+    <t>Table C.10</t>
+  </si>
+  <si>
+    <t>do/tables/tabC10.do</t>
+  </si>
+  <si>
+    <t>Table C.11</t>
+  </si>
+  <si>
+    <t>do/tables/tabC11.do</t>
+  </si>
+  <si>
+    <t>142</t>
+  </si>
+  <si>
+    <t>Table C.12</t>
+  </si>
+  <si>
+    <t>do/tables/tabC12.do</t>
+  </si>
+  <si>
+    <t>Table D.1</t>
+  </si>
+  <si>
+    <t>do/tables/tabD1.do</t>
+  </si>
+  <si>
+    <t>186</t>
+  </si>
+  <si>
+    <t>Table D.2</t>
+  </si>
+  <si>
+    <t>do/tables/tabD2.do</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>Table D.3</t>
+  </si>
+  <si>
+    <t>do/tables/tabD3.do</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>Table E.1</t>
+  </si>
+  <si>
+    <t>286</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>n/a</t>
   </si>
 </sst>
 </file>
@@ -89,7 +551,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -99,6 +561,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,12 +899,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="56" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
@@ -449,7 +914,7 @@
     <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,49 +925,836 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
-      </c>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" t="s">
+        <v>81</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D37" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" t="s">
+        <v>87</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>89</v>
+      </c>
+      <c r="B39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" t="s">
+        <v>70</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D41" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>98</v>
+      </c>
+      <c r="B43" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>101</v>
+      </c>
+      <c r="B44" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D44" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D45" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>106</v>
+      </c>
+      <c r="B46" t="s">
+        <v>107</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D46" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>108</v>
+      </c>
+      <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D47" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>111</v>
+      </c>
+      <c r="B48" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>114</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D49" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>115</v>
+      </c>
+      <c r="B50" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>118</v>
+      </c>
+      <c r="B51" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>120</v>
+      </c>
+      <c r="B52" t="s">
+        <v>121</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" t="s">
+        <v>124</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D53" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>126</v>
+      </c>
+      <c r="B54" t="s">
+        <v>127</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D54" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>129</v>
+      </c>
+      <c r="B55" t="s">
+        <v>130</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D55" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>131</v>
+      </c>
+      <c r="B56" t="s">
+        <v>132</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D56" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>134</v>
+      </c>
+      <c r="B57" t="s">
+        <v>135</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D57" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>136</v>
+      </c>
+      <c r="B58" t="s">
+        <v>137</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D58" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>138</v>
+      </c>
+      <c r="B59" t="s">
+        <v>139</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D59" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>140</v>
+      </c>
+      <c r="B60" t="s">
+        <v>141</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D60" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>143</v>
+      </c>
+      <c r="B61" t="s">
+        <v>144</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D61" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>145</v>
+      </c>
+      <c r="B62" t="s">
+        <v>146</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D62" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>148</v>
+      </c>
+      <c r="B63" t="s">
+        <v>149</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D63" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>151</v>
+      </c>
+      <c r="B64" t="s">
+        <v>152</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D64" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>154</v>
+      </c>
+      <c r="B65" t="s">
+        <v>70</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D65" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="1"/>
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="2"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C68" s="3"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C69" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>